<commit_message>
Changing port in server
</commit_message>
<xml_diff>
--- a/pos_database.xlsx
+++ b/pos_database.xlsx
@@ -436,7 +436,7 @@
         <v>25</v>
       </c>
       <c r="E2">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>50</v>
       </c>
       <c r="E3">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -470,7 +470,7 @@
         <v>100</v>
       </c>
       <c r="E4">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -482,7 +482,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -764,16 +764,226 @@
         <v>275</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>R1780088242889</v>
+      </c>
+      <c r="B9" t="str">
+        <v>05/30/2026</v>
+      </c>
+      <c r="C9" t="str">
+        <v>4:57:22 AM</v>
+      </c>
+      <c r="D9" t="str">
+        <v>cashier</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Cheese Bar</v>
+      </c>
+      <c r="F9" t="str">
+        <v>DRY-001</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Dairy Products</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>25</v>
+      </c>
+      <c r="J9">
+        <v>25</v>
+      </c>
+      <c r="K9">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>R1780088242889</v>
+      </c>
+      <c r="B10" t="str">
+        <v>05/30/2026</v>
+      </c>
+      <c r="C10" t="str">
+        <v>4:57:22 AM</v>
+      </c>
+      <c r="D10" t="str">
+        <v>cashier</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Burger Buns</v>
+      </c>
+      <c r="F10" t="str">
+        <v>BRD-001</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Bread &amp; Buns</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>50</v>
+      </c>
+      <c r="J10">
+        <v>50</v>
+      </c>
+      <c r="K10">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>R1780088242889</v>
+      </c>
+      <c r="B11" t="str">
+        <v>05/30/2026</v>
+      </c>
+      <c r="C11" t="str">
+        <v>4:57:22 AM</v>
+      </c>
+      <c r="D11" t="str">
+        <v>cashier</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Kogi</v>
+      </c>
+      <c r="F11" t="str">
+        <v>MET-001</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Meat Products</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>100</v>
+      </c>
+      <c r="J11">
+        <v>100</v>
+      </c>
+      <c r="K11">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>R1780088415285</v>
+      </c>
+      <c r="B12" t="str">
+        <v>05/30/2026</v>
+      </c>
+      <c r="C12" t="str">
+        <v>5:00:15 AM</v>
+      </c>
+      <c r="D12" t="str">
+        <v>cashier</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Cheese Bar</v>
+      </c>
+      <c r="F12" t="str">
+        <v>DRY-001</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Dairy Products</v>
+      </c>
+      <c r="H12">
+        <v>3</v>
+      </c>
+      <c r="I12">
+        <v>25</v>
+      </c>
+      <c r="J12">
+        <v>75</v>
+      </c>
+      <c r="K12">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>R1780088415285</v>
+      </c>
+      <c r="B13" t="str">
+        <v>05/30/2026</v>
+      </c>
+      <c r="C13" t="str">
+        <v>5:00:15 AM</v>
+      </c>
+      <c r="D13" t="str">
+        <v>cashier</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Burger Buns</v>
+      </c>
+      <c r="F13" t="str">
+        <v>BRD-001</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Bread &amp; Buns</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>50</v>
+      </c>
+      <c r="J13">
+        <v>50</v>
+      </c>
+      <c r="K13">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>R1780088415285</v>
+      </c>
+      <c r="B14" t="str">
+        <v>05/30/2026</v>
+      </c>
+      <c r="C14" t="str">
+        <v>5:00:15 AM</v>
+      </c>
+      <c r="D14" t="str">
+        <v>cashier</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Kogi</v>
+      </c>
+      <c r="F14" t="str">
+        <v>MET-001</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Meat Products</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>100</v>
+      </c>
+      <c r="J14">
+        <v>100</v>
+      </c>
+      <c r="K14">
+        <v>225</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K14"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -907,16 +1117,56 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>R1780088242889</v>
+      </c>
+      <c r="B7" t="str">
+        <v>05/30/2026</v>
+      </c>
+      <c r="C7" t="str">
+        <v>4:57:22 AM</v>
+      </c>
+      <c r="D7" t="str">
+        <v>cashier</v>
+      </c>
+      <c r="E7">
+        <v>175</v>
+      </c>
+      <c r="F7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>R1780088415285</v>
+      </c>
+      <c r="B8" t="str">
+        <v>05/30/2026</v>
+      </c>
+      <c r="C8" t="str">
+        <v>5:00:15 AM</v>
+      </c>
+      <c r="D8" t="str">
+        <v>cashier</v>
+      </c>
+      <c r="E8">
+        <v>225</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1034,9 +1284,38 @@
         <v>100</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>05/30/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>4:54:38 AM</v>
+      </c>
+      <c r="C5" t="str">
+        <v>MET-001</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Kogi</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Meat Products</v>
+      </c>
+      <c r="F5">
+        <v>9</v>
+      </c>
+      <c r="G5">
+        <v>8</v>
+      </c>
+      <c r="H5">
+        <v>17</v>
+      </c>
+      <c r="I5">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>